<commit_message>
V3 final + 꿈이든 + 번역기
</commit_message>
<xml_diff>
--- a/data/elementary.xlsx
+++ b/data/elementary.xlsx
@@ -5,7 +5,7 @@
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\특수학급지도 - V3\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\특수학급지도 - V3 final + 꿈이든 + 번역기\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
@@ -21,184 +21,43 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="233">
   <x:si>
-    <x:t>3명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-310-4695</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-363-1526</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 배곧4로 94-39</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 월곶해안로 69</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 능곡중앙로 22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 황고개로 567</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 목감둘레로 109</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 장곡로 70번길 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 목감초등길 49</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 배곧 4로 44-5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 신천로 7번길 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 목감남서로 68</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 배곧1로 28-25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>한국글로벌중학구/ 소래중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 계수로 203</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7096-7801</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8063-7873</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-503-1538</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8044-1261</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 해송십리로 472-30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 서울대학로 150-17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 대은로 104번길 29-10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 정왕대로 143번길 15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 옥구천동로 433-25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 하중로 209번길 10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 정왕천로427번길 30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 정왕대로 53번길 14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 수인로3247번길 59</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 정왕대로118번길 27</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 수인로 3413번길 34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 신현로 202번길 31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>13명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7096-7706</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-503-0560</x:t>
-  </x:si>
-  <x:si>
-    <x:t>한여울초등학교(복합특수)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-1683</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-2204</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-364-7903</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-0802</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 군자로 539</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-2707</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-490-8204</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 은행고길 18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8063-2903</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7014-4072</x:t>
+    <x:t>⊙연성초등학교 학구 중 목감동 1~2통, 3통 4반~6반은 목감중학구 및 안산시 안산중학구와 공동학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수/순회/일반)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥능곡초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧라온초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥도원초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧라라초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧한울초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>소래중학구/연성중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥가온초등학교</x:t>
   </x:si>
   <x:si>
     <x:t>031-8042-0004</x:t>
   </x:si>
   <x:si>
+    <x:t>031-317-2701</x:t>
+  </x:si>
+  <x:si>
     <x:t>070-7097-0204</x:t>
   </x:si>
   <x:si>
-    <x:t>031-317-2701</x:t>
-  </x:si>
-  <x:si>
-    <x:t>-</x:t>
-  </x:si>
-  <x:si>
-    <x:t>공립</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 주소</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 비고</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7096-6083</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7015-4404</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-0603</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-2915</x:t>
-  </x:si>
-  <x:si>
-    <x:t>성인 · 주부 · 어르신</x:t>
+    <x:t>070-7014-8703</x:t>
   </x:si>
   <x:si>
     <x:t>경기도 시흥시 포도원로 88</x:t>
@@ -210,44 +69,17 @@
     <x:t>031-412-4300</x:t>
   </x:si>
   <x:si>
-    <x:t>070-7014-8703</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-503-1020</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7096-6872</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-312-3600</x:t>
-  </x:si>
-  <x:si>
-    <x:t>복특 6학급/ 시간제 2학급</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-4648-5770</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7016-3005</x:t>
+    <x:t>031-8042-2502</x:t>
   </x:si>
   <x:si>
     <x:t>한국글로벌중학구
 /소래중학구</x:t>
   </x:si>
   <x:si>
-    <x:t>031-8042-2502</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-364-3410</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8099-5900</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8042-0700</x:t>
-  </x:si>
-  <x:si>
-    <x:t>⊙연성초등학교 학구 중 목감동 1~2통, 3통 4반~6반은 목감중학구 및 안산시 안산중학구와 공동학구</x:t>
+    <x:t>070-7096-6083</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-0603</x:t>
   </x:si>
   <x:si>
     <x:t>⊙도창초등학교 학구 중 매화동 5통, 매화동 20~22통은 시흥매화중학구와 공동학구
@@ -255,472 +87,640 @@
 ⊙도창초등학교 학구 중 과림동 1통(노무저리 제외),  과림동 2통은 광명시 광명중학군과 공동학구</x:t>
   </x:si>
   <x:si>
-    <x:t>소래중학구/연성중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥가온초등학교</x:t>
-  </x:si>
-  <x:si>
     <x:t>경기도 시흥시 나분들길 44</x:t>
   </x:si>
   <x:si>
+    <x:t>031-8042-0700</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8099-5900</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-434-6152</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-364-3410</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥신일초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧누리초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥매화초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥은행초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥월곶초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>목감중학구/조남중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧해솔초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시화나래초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥장현초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>한국글로벌중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>군서미래국제학교(초)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7015-4404</x:t>
+  </x:si>
+  <x:si>
+    <x:t>성인 · 주부 · 어르신</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-2915</x:t>
+  </x:si>
+  <x:si>
+    <x:t>복특 6학급/ 시간제 2학급</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8032-6504</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8099-9703</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-363-5904</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-365-8003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8040-6505</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 역전로 455</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(복합특수/시간제/일반)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-500-0601</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 포도원로 39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 대골안길 31</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8085-7004</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7096-7772</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-503-0560</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8063-7873</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7096-7706</x:t>
+  </x:si>
+  <x:si>
+    <x:t>한여울초등학교(복합특수)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7096-7801</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-503-1538</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8044-1261</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-1108</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-1683</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-1303</x:t>
+  </x:si>
+  <x:si>
+    <x:t>계수초등학교 학구 중 계수동은 부천시 소사옥길중학군과 공동학구</x:t>
+  </x:si>
+  <x:si>
     <x:t>경기도 시흥시 승지로 110</x:t>
   </x:si>
   <x:si>
+    <x:t>031-364-7903</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-0802</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-312-3600</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-310-4695</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-363-1526</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-490-8204</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-2707</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 은행고길 18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-4648-5770</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7014-4072</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 군자로 539</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 옥터로 33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-2576</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 능곡군자로 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-2302</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 매화1로 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-363-3003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>목감중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>정왕중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥매화중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>소래중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>승지초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>하중초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>은계초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21/ 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>은빛초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>진말초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>장곡중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>소래초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대야초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>생금초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>도일초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>연성초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>산현초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 목감초등길 49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 목감둘레로 109</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 장곡로 70번길 12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 신천로 7번길 12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 배곧1로 28-25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 배곧 4로 44-5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 목감남서로 68</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 서울대학로 255</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 대은로103번길 24</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">경기도 시흥시 은행동 663 </x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 중심상가로 257</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 죽율로 45-42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 호현로 27번길 14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 군자로465번길 7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 군서마을로 101</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 시청로80번길 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 목감둘레로 229-9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 거북섬남로 70</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 큰솔로 7번길 10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 월곶중앙로 18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 대은로 16-29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 장현능곡로 33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 수인로2793번길 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 월곶해안로 69</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 능곡중앙로 22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 배곧4로 94-39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 황고개로 567</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 서울대학로 150-17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 해송십리로 472-30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 대은로 104번길 29-10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 정왕대로 143번길 15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 정왕천로427번길 30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 정왕대로 53번길 14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 수인로3247번길 59</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 하중로 209번길 10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 옥구천동로 433-25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 수인로 3413번길 34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 정왕대로118번길 27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 신현로 202번길 31</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-8063-2903</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7016-3005</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-2204</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경기도 시흥시 계수로 203</x:t>
+  </x:si>
+  <x:si>
+    <x:t>한국글로벌중학구/ 소래중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7097-1553</x:t>
+  </x:si>
+  <x:si>
+    <x:t>031-494-4167</x:t>
+  </x:si>
+  <x:si>
     <x:t>경기도 시흥시 역전로 369</x:t>
   </x:si>
   <x:si>
-    <x:t>경기도 시흥시 옥터로 33</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-2576</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 능곡군자로 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-2302</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-363-3003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 매화1로 6</x:t>
-  </x:si>
-  <x:si>
     <x:t>031-364-1700</x:t>
   </x:si>
   <x:si>
-    <x:t>070-7097-1108</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-494-4167</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-1553</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8032-6504</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-434-6152</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7097-1303</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8085-7004</x:t>
-  </x:si>
-  <x:si>
-    <x:t>070-7096-7772</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8099-9703</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-8040-6505</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-363-5904</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 역전로 455</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-365-8003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>031-500-0601</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(복합특수/시간제/일반)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 대골안길 31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 포도원로 39</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥장현초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>한국글로벌중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>군서미래국제학교(초)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧누리초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥신일초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥매화초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>계수초등학교 학구 중 계수동은 부천시 소사옥길중학군과 공동학구</x:t>
+    <x:t>031-503-1020</x:t>
+  </x:si>
+  <x:si>
+    <x:t>070-7096-6872</x:t>
+  </x:si>
+  <x:si>
+    <x:t>경도</x:t>
+  </x:si>
+  <x:si>
+    <x:t>유</x:t>
+  </x:si>
+  <x:si>
+    <x:t>위도</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-</x:t>
+  </x:si>
+  <x:si>
+    <x:t>공립</x:t>
+  </x:si>
+  <x:si>
+    <x:t>⊙목감초등학교 학구 중 목감동 4통, 6통은 안산중학구와 공동학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>진영초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>연성중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>신천초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15/ 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥능곡중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>월곶중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>월포초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수/순회)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웃터골초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>송운초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>서촌초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>포리초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>금모래초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>목감초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24/ 12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>도창초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>군서초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>냉정초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥터초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>함현초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>계수초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3학기제</x:t>
+  </x:si>
+  <x:si>
+    <x:t>군자초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>조남초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>운흥초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>배곧초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>장곡초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시흥초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시화중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시화초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>서해초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>군자중학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>정왕초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>검바위초등학교</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 19명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 16명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 10명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 특수/순회학급수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>보조인력 배치 유/무</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 2학급)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 6명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 14명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 13명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 5명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 21명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 1학급)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 8명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 4학급)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 22명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 3학급)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 4명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 2명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 7명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 18명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 17명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 9명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 11명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 15명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 20명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(특수 : 23명)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 연락처</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 학교명</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 학교설립별</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16/ 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>일반학급 배치 학생 수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>특수/순회학급 배치 학생 수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5명</x:t>
   </x:si>
   <x:si>
     <x:t>1명</x:t>
   </x:si>
   <x:si>
-    <x:t>서해초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>정왕초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>검바위초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>정왕중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥매화중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>목감중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>하중초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>승지초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>소래중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>연성초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>은빛초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>산현초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>은계초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21/ 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>진말초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>소래초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>대야초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>장곡중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>생금초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>도일초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>연성중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15/ 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>신천초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥능곡중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>진영초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웃터골초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수/순회)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>월곶중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>월포초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>포리초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>송운초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>서촌초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>도창초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>목감초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>금모래초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>군서초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24/ 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>함현초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>냉정초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>계수초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥터초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>군자초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3학기제</x:t>
-  </x:si>
-  <x:si>
-    <x:t>장곡초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>운흥초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16/ 2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>조남초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시화초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시화중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>군자중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥은행초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧해솔초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥월곶초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시화나래초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>목감중학구/조남중학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 서울대학로 255</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 대은로103번길 24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 호현로 27번길 14</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">경기도 시흥시 은행동 663 </x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 죽율로 45-42</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 중심상가로 257</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 시청로80번길 5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 거북섬남로 70</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 목감둘레로 229-9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 군자로465번길 7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 군서마을로 101</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 월곶중앙로 18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 수인로2793번길 6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 큰솔로 7번길 10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 대은로 16-29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경기도 시흥시 장현능곡로 33</x:t>
-  </x:si>
-  <x:si>
-    <x:t>⊙목감초등학교 학구 중 목감동 4통, 6통은 안산중학구와 공동학구</x:t>
-  </x:si>
-  <x:si>
-    <x:t>유</x:t>
-  </x:si>
-  <x:si>
-    <x:t>경도</x:t>
-  </x:si>
-  <x:si>
-    <x:t>위도</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수/순회/일반)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧라온초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥능곡초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시흥도원초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧라라초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>배곧한울초등학교</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 19명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 2학급)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 6명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 13명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 16명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 10명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 특수/순회학급수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>보조인력 배치 유/무</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 14명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 8명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 21명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 5명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 1학급)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 3학급)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 4명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 4학급)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 22명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 7명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 18명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 2명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 17명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 9명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 11명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 15명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 20명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(특수 : 23명)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5명</x:t>
-  </x:si>
-  <x:si>
     <x:t>10명</x:t>
   </x:si>
   <x:si>
+    <x:t>4명</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 비고</x:t>
+  </x:si>
+  <x:si>
     <x:t>2명</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> 연락처</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 학교명</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 학교설립별</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4명</x:t>
-  </x:si>
-  <x:si>
-    <x:t>일반학급 배치 학생 수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>특수/순회학급 배치 학생 수</x:t>
+    <x:t xml:space="preserve"> 학구</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13명</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve"> 주소</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7명</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3명</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1135,73 +1135,74 @@
     <x:col min="6" max="6" width="27.62890625" customWidth="1"/>
     <x:col min="7" max="7" width="24.55078125" bestFit="1" customWidth="1"/>
     <x:col min="8" max="8" width="19.9921875" bestFit="1" customWidth="1"/>
+    <x:col min="11" max="12" width="11.51171875" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:12">
       <x:c r="A1" t="s">
+        <x:v>217</x:v>
+      </x:c>
+      <x:c r="B1" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="C1" t="s">
         <x:v>228</x:v>
       </x:c>
-      <x:c r="B1" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="C1" t="s">
-        <x:v>52</x:v>
-      </x:c>
       <x:c r="D1" t="s">
-        <x:v>53</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E1" t="s">
-        <x:v>227</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="F1" t="s">
-        <x:v>204</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="G1" t="s">
-        <x:v>232</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="H1" t="s">
-        <x:v>231</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="I1" t="s">
-        <x:v>205</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="J1" t="s">
-        <x:v>54</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="K1" t="s">
-        <x:v>191</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="L1" t="s">
-        <x:v>190</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:12" ht="65.5">
       <x:c r="A2" t="s">
-        <x:v>116</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B2" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D2" t="s">
-        <x:v>28</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E2" t="s">
-        <x:v>18</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F2" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G2" t="s">
-        <x:v>208</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H2" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I2" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K2">
         <x:v>37.432746760000001</x:v>
@@ -1212,34 +1213,34 @@
     </x:row>
     <x:row r="3" spans="1:12">
       <x:c r="A3" t="s">
-        <x:v>154</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="B3" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C3" t="s">
-        <x:v>107</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" t="s">
-        <x:v>15</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E3" t="s">
-        <x:v>19</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F3" t="s">
-        <x:v>210</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G3" t="s">
-        <x:v>212</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H3" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I3" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J3" t="s">
-        <x:v>112</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="K3">
         <x:v>37.453471950000001</x:v>
@@ -1250,31 +1251,31 @@
     </x:row>
     <x:row r="4" spans="1:12">
       <x:c r="A4" t="s">
-        <x:v>108</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B4" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C4" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D4" t="s">
-        <x:v>182</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E4" t="s">
-        <x:v>2</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F4" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="G4" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="H4" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I4" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K4">
         <x:v>37.34626506</x:v>
@@ -1285,31 +1286,31 @@
     </x:row>
     <x:row r="5" spans="1:12">
       <x:c r="A5" t="s">
-        <x:v>150</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C5" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D5" t="s">
-        <x:v>26</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E5" t="s">
-        <x:v>71</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F5" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G5" t="s">
-        <x:v>214</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="H5" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I5" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K5">
         <x:v>37.347420020000001</x:v>
@@ -1320,31 +1321,31 @@
     </x:row>
     <x:row r="6" spans="1:12">
       <x:c r="A6" t="s">
-        <x:v>157</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B6" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C6" t="s">
-        <x:v>166</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>41</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E6" t="s">
-        <x:v>68</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F6" t="s">
-        <x:v>213</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="G6" t="s">
-        <x:v>208</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H6" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I6" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K6">
         <x:v>37.343899370000003</x:v>
@@ -1355,31 +1356,31 @@
     </x:row>
     <x:row r="7" spans="1:12" ht="65.5">
       <x:c r="A7" t="s">
-        <x:v>149</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B7" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D7" t="s">
-        <x:v>186</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E7" t="s">
-        <x:v>57</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F7" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G7" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="H7" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I7" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K7">
         <x:v>37.441589</x:v>
@@ -1390,31 +1391,31 @@
     </x:row>
     <x:row r="8" spans="1:12">
       <x:c r="A8" t="s">
-        <x:v>153</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B8" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C8" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>81</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E8" t="s">
-        <x:v>74</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F8" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G8" t="s">
-        <x:v>198</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="H8" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I8" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K8">
         <x:v>37.357741859999997</x:v>
@@ -1425,31 +1426,31 @@
     </x:row>
     <x:row r="9" spans="1:12">
       <x:c r="A9" t="s">
-        <x:v>130</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B9" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C9" t="s">
-        <x:v>14</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>104</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E9" t="s">
-        <x:v>86</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F9" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G9" t="s">
-        <x:v>202</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="H9" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I9" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K9">
         <x:v>37.446825369999999</x:v>
@@ -1460,19 +1461,19 @@
     </x:row>
     <x:row r="10" spans="1:12">
       <x:c r="A10" t="s">
-        <x:v>134</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C10" t="s">
-        <x:v>166</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>181</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="E10" t="s">
-        <x:v>90</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="F10" s="2">
         <x:v>46054</x:v>
@@ -1481,13 +1482,13 @@
         <x:v>46268</x:v>
       </x:c>
       <x:c r="H10" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I10" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J10" t="s">
-        <x:v>141</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="K10">
         <x:v>37.349119160000001</x:v>
@@ -1498,22 +1499,22 @@
     </x:row>
     <x:row r="11" spans="1:12" ht="409.5">
       <x:c r="A11" t="s">
-        <x:v>147</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B11" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D11" t="s">
-        <x:v>184</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="E11" t="s">
-        <x:v>85</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F11" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="G11">
         <x:v>0</x:v>
@@ -1522,10 +1523,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J11" s="1" t="s">
-        <x:v>76</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K11">
         <x:v>37.406893609999997</x:v>
@@ -1536,34 +1537,34 @@
     </x:row>
     <x:row r="12" spans="1:12">
       <x:c r="A12" t="s">
-        <x:v>148</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B12" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C12" t="s">
-        <x:v>119</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D12" t="s">
-        <x:v>9</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E12" t="s">
-        <x:v>91</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="F12" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G12" t="s">
-        <x:v>203</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="H12" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I12" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J12" t="s">
-        <x:v>188</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="K12">
         <x:v>37.386862639999997</x:v>
@@ -1574,31 +1575,31 @@
     </x:row>
     <x:row r="13" spans="1:12">
       <x:c r="A13" t="s">
-        <x:v>109</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B13" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C13" t="s">
-        <x:v>132</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D13" t="s">
-        <x:v>20</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="E13" t="s">
-        <x:v>45</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F13" t="s">
-        <x:v>213</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="G13" t="s">
-        <x:v>208</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I13" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K13">
         <x:v>37.382653580000003</x:v>
@@ -1609,31 +1610,31 @@
     </x:row>
     <x:row r="14" spans="1:12">
       <x:c r="A14" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B14" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="C14" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="D14" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="E14" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="F14" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="G14" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="B14" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="C14" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="D14" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="E14" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F14" t="s">
-        <x:v>210</x:v>
-      </x:c>
-      <x:c r="G14" t="s">
-        <x:v>200</x:v>
-      </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I14" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K14">
         <x:v>37.369258219999999</x:v>
@@ -1644,31 +1645,31 @@
     </x:row>
     <x:row r="15" spans="1:12">
       <x:c r="A15" t="s">
-        <x:v>193</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C15" t="s">
-        <x:v>132</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D15" t="s">
-        <x:v>3</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E15" t="s">
-        <x:v>92</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F15" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G15" t="s">
-        <x:v>222</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I15" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K15">
         <x:v>37.372575730000001</x:v>
@@ -1679,31 +1680,31 @@
     </x:row>
     <x:row r="16" spans="1:12">
       <x:c r="A16" t="s">
-        <x:v>160</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B16" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C16" t="s">
-        <x:v>132</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D16" t="s">
-        <x:v>10</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E16" t="s">
-        <x:v>97</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F16" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G16" t="s">
-        <x:v>221</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I16" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K16">
         <x:v>37.376015750000001</x:v>
@@ -1714,31 +1715,31 @@
     </x:row>
     <x:row r="17" spans="1:12">
       <x:c r="A17" t="s">
-        <x:v>197</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B17" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C17" t="s">
-        <x:v>132</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D17" t="s">
-        <x:v>13</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E17" t="s">
-        <x:v>62</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F17" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G17" t="s">
-        <x:v>198</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="H17" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I17" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K17">
         <x:v>37.360501769999999</x:v>
@@ -1749,31 +1750,31 @@
     </x:row>
     <x:row r="18" spans="1:12">
       <x:c r="A18" t="s">
-        <x:v>168</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B18" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C18" t="s">
-        <x:v>132</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D18" t="s">
-        <x:v>21</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E18" t="s">
-        <x:v>17</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F18" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G18" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H18" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I18" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K18">
         <x:v>37.360535210000002</x:v>
@@ -1784,31 +1785,31 @@
     </x:row>
     <x:row r="19" spans="1:12">
       <x:c r="A19" t="s">
-        <x:v>125</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B19" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C19" t="s">
-        <x:v>171</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D19" t="s">
-        <x:v>12</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E19" t="s">
-        <x:v>98</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F19" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G19" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="H19" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I19" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K19">
         <x:v>37.37494805</x:v>
@@ -1819,31 +1820,31 @@
     </x:row>
     <x:row r="20" spans="1:12">
       <x:c r="A20" t="s">
-        <x:v>133</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C20" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D20" t="s">
-        <x:v>176</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E20" t="s">
-        <x:v>69</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="F20" t="s">
-        <x:v>210</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G20" t="s">
-        <x:v>209</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="H20" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="I20" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K20">
         <x:v>37.350397829999999</x:v>
@@ -1854,31 +1855,31 @@
     </x:row>
     <x:row r="21" spans="1:12">
       <x:c r="A21" t="s">
-        <x:v>146</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C21" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D21" t="s">
-        <x:v>29</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E21" t="s">
-        <x:v>46</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F21" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G21" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="H21" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I21" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K21">
         <x:v>37.349460039999997</x:v>
@@ -1889,34 +1890,34 @@
     </x:row>
     <x:row r="22" spans="1:12">
       <x:c r="A22" t="s">
-        <x:v>114</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C22" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D22" t="s">
-        <x:v>27</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E22" t="s">
-        <x:v>93</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F22" s="2">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="G22" t="s">
-        <x:v>162</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="H22" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I22" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J22" t="s">
-        <x:v>192</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K22">
         <x:v>37.356151019999999</x:v>
@@ -1927,31 +1928,31 @@
     </x:row>
     <x:row r="23" spans="1:12">
       <x:c r="A23" t="s">
-        <x:v>129</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C23" t="s">
-        <x:v>122</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D23" t="s">
-        <x:v>174</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E23" t="s">
-        <x:v>37</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F23" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G23" t="s">
-        <x:v>207</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H23" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I23" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K23">
         <x:v>37.443772459999998</x:v>
@@ -1962,31 +1963,31 @@
     </x:row>
     <x:row r="24" spans="1:12">
       <x:c r="A24" t="s">
-        <x:v>145</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B24" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C24" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D24" t="s">
-        <x:v>24</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E24" t="s">
-        <x:v>102</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F24" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G24" t="s">
-        <x:v>206</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H24" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I24" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K24">
         <x:v>35.228763190000002</x:v>
@@ -1997,31 +1998,31 @@
     </x:row>
     <x:row r="25" spans="1:12">
       <x:c r="A25" t="s">
-        <x:v>121</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B25" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C25" t="s">
-        <x:v>138</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D25" t="s">
-        <x:v>80</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E25" t="s">
-        <x:v>73</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F25" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G25" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H25" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I25" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K25">
         <x:v>37.372313550000001</x:v>
@@ -2032,31 +2033,31 @@
     </x:row>
     <x:row r="26" spans="1:12">
       <x:c r="A26" t="s">
-        <x:v>170</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B26" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C26" t="s">
-        <x:v>165</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D26" t="s">
-        <x:v>179</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E26" t="s">
-        <x:v>72</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F26" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G26" t="s">
-        <x:v>206</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H26" t="s">
-        <x:v>32</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="I26" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K26">
         <x:v>37.320716019999999</x:v>
@@ -2067,31 +2068,31 @@
     </x:row>
     <x:row r="27" spans="1:12">
       <x:c r="A27" t="s">
-        <x:v>164</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B27" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C27" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D27" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="D27" t="s">
-        <x:v>185</x:v>
-      </x:c>
       <x:c r="E27" t="s">
-        <x:v>35</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F27" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G27" t="s">
-        <x:v>221</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H27" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I27" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K27">
         <x:v>37.339255610000002</x:v>
@@ -2102,31 +2103,31 @@
     </x:row>
     <x:row r="28" spans="1:12">
       <x:c r="A28" t="s">
-        <x:v>78</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B28" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C28" t="s">
-        <x:v>131</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D28" t="s">
-        <x:v>187</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="E28" t="s">
-        <x:v>88</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="F28" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G28" t="s">
-        <x:v>223</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I28" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K28">
         <x:v>37.37378717</x:v>
@@ -2137,31 +2138,31 @@
     </x:row>
     <x:row r="29" spans="1:12">
       <x:c r="A29" t="s">
-        <x:v>194</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B29" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C29" t="s">
-        <x:v>138</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D29" t="s">
-        <x:v>5</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E29" t="s">
-        <x:v>65</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F29" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G29" t="s">
-        <x:v>203</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I29" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K29">
         <x:v>37.365372309999998</x:v>
@@ -2172,31 +2173,31 @@
     </x:row>
     <x:row r="30" spans="1:12">
       <x:c r="A30" t="s">
-        <x:v>195</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B30" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C30" t="s">
-        <x:v>122</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D30" t="s">
-        <x:v>30</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="E30" t="s">
-        <x:v>89</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F30" t="s">
-        <x:v>210</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G30" t="s">
-        <x:v>212</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I30" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K30">
         <x:v>37.440093009999998</x:v>
@@ -2207,31 +2208,31 @@
     </x:row>
     <x:row r="31" spans="1:12">
       <x:c r="A31" t="s">
-        <x:v>111</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B31" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C31" t="s">
-        <x:v>118</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D31" t="s">
-        <x:v>87</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E31" t="s">
-        <x:v>47</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F31" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G31" t="s">
-        <x:v>218</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="H31" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I31" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K31">
         <x:v>37.416300909999997</x:v>
@@ -2242,31 +2243,31 @@
     </x:row>
     <x:row r="32" spans="1:12">
       <x:c r="A32" t="s">
-        <x:v>110</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B32" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C32" t="s">
-        <x:v>122</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D32" t="s">
-        <x:v>11</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E32" t="s">
-        <x:v>61</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F32" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G32" t="s">
-        <x:v>207</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H32" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I32" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K32">
         <x:v>37.433075209999998</x:v>
@@ -2277,31 +2278,31 @@
     </x:row>
     <x:row r="33" spans="1:12">
       <x:c r="A33" t="s">
-        <x:v>169</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B33" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C33" t="s">
-        <x:v>142</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="D33" t="s">
-        <x:v>4</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E33" t="s">
-        <x:v>39</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F33" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G33" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="H33" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I33" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K33">
         <x:v>37.391718959999999</x:v>
@@ -2312,31 +2313,31 @@
     </x:row>
     <x:row r="34" spans="1:12" ht="65.5">
       <x:c r="A34" t="s">
-        <x:v>167</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B34" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D34" t="s">
-        <x:v>22</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E34" t="s">
-        <x:v>48</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F34" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G34" t="s">
-        <x:v>216</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="H34" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I34" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K34">
         <x:v>37.442591470000004</x:v>
@@ -2347,31 +2348,31 @@
     </x:row>
     <x:row r="35" spans="1:12">
       <x:c r="A35" t="s">
-        <x:v>106</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B35" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C35" t="s">
-        <x:v>131</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D35" t="s">
-        <x:v>178</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E35" t="s">
-        <x:v>1</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="F35" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G35" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="H35" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="I35" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K35">
         <x:v>37.381790879999997</x:v>
@@ -2382,31 +2383,31 @@
     </x:row>
     <x:row r="36" spans="1:12">
       <x:c r="A36" t="s">
-        <x:v>156</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B36" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C36" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D36" t="s">
-        <x:v>23</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E36" t="s">
-        <x:v>58</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F36" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G36" t="s">
-        <x:v>216</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="H36" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I36" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K36">
         <x:v>33.479625749999997</x:v>
@@ -2417,31 +2418,31 @@
     </x:row>
     <x:row r="37" spans="1:12">
       <x:c r="A37" t="s">
-        <x:v>137</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B37" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C37" t="s">
-        <x:v>122</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D37" t="s">
-        <x:v>60</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E37" t="s">
-        <x:v>38</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="F37" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G37" t="s">
-        <x:v>220</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H37" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I37" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K37">
         <x:v>37.43524335</x:v>
@@ -2452,34 +2453,34 @@
     </x:row>
     <x:row r="38" spans="1:12">
       <x:c r="A38" t="s">
-        <x:v>123</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B38" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C38" t="s">
-        <x:v>119</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D38" t="s">
-        <x:v>79</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E38" t="s">
-        <x:v>63</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F38" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G38" t="s">
-        <x:v>207</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="H38" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I38" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J38" t="s">
-        <x:v>75</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K38">
         <x:v>37.387563890000003</x:v>
@@ -2490,31 +2491,31 @@
     </x:row>
     <x:row r="39" spans="1:12">
       <x:c r="A39" t="s">
-        <x:v>155</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B39" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C39" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D39" t="s">
-        <x:v>82</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E39" t="s">
-        <x:v>56</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F39" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G39" t="s">
-        <x:v>221</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H39" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I39" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K39">
         <x:v>37.345110460000001</x:v>
@@ -2525,31 +2526,31 @@
     </x:row>
     <x:row r="40" spans="1:12">
       <x:c r="A40" t="s">
-        <x:v>161</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B40" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C40" t="s">
-        <x:v>171</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D40" t="s">
-        <x:v>7</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E40" t="s">
-        <x:v>99</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F40" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G40" t="s">
-        <x:v>206</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H40" t="s">
-        <x:v>225</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="I40" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K40">
         <x:v>37.372765039999997</x:v>
@@ -2560,31 +2561,31 @@
     </x:row>
     <x:row r="41" spans="1:12" ht="65.5">
       <x:c r="A41" t="s">
-        <x:v>140</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B41" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D41" t="s">
-        <x:v>44</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E41" t="s">
-        <x:v>34</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="F41" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G41" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="H41" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I41" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K41">
         <x:v>37.439720010000002</x:v>
@@ -2595,31 +2596,31 @@
     </x:row>
     <x:row r="42" spans="1:12">
       <x:c r="A42" t="s">
-        <x:v>143</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B42" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C42" t="s">
-        <x:v>142</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="D42" t="s">
-        <x:v>183</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E42" t="s">
-        <x:v>42</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F42" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G42" t="s">
-        <x:v>219</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="H42" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I42" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K42">
         <x:v>37.387488849999997</x:v>
@@ -2630,34 +2631,34 @@
     </x:row>
     <x:row r="43" spans="1:12" ht="65.5">
       <x:c r="A43" t="s">
-        <x:v>126</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B43" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D43" t="s">
-        <x:v>173</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E43" t="s">
-        <x:v>96</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F43" s="2">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="G43" t="s">
-        <x:v>136</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="H43" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I43" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J43" t="s">
-        <x:v>192</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K43">
         <x:v>37.44773309</x:v>
@@ -2668,31 +2669,31 @@
     </x:row>
     <x:row r="44" spans="1:12" ht="65.5">
       <x:c r="A44" t="s">
-        <x:v>124</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B44" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="C44" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D44" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E44" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C44" s="1" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="D44" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="E44" t="s">
-        <x:v>95</x:v>
-      </x:c>
       <x:c r="F44" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G44" t="s">
-        <x:v>208</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="H44" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I44" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K44">
         <x:v>37.434280770000001</x:v>
@@ -2703,31 +2704,31 @@
     </x:row>
     <x:row r="45" spans="1:12">
       <x:c r="A45" t="s">
-        <x:v>159</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B45" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C45" t="s">
-        <x:v>131</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D45" t="s">
-        <x:v>8</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E45" t="s">
-        <x:v>55</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F45" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G45" t="s">
-        <x:v>206</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H45" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I45" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K45">
         <x:v>37.381523569999999</x:v>
@@ -2738,34 +2739,34 @@
     </x:row>
     <x:row r="46" spans="1:12">
       <x:c r="A46" t="s">
-        <x:v>115</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B46" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C46" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D46" t="s">
-        <x:v>177</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="E46" t="s">
-        <x:v>16</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F46" s="2">
         <x:v>46082</x:v>
       </x:c>
       <x:c r="G46" t="s">
-        <x:v>127</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="H46" t="s">
-        <x:v>0</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="I46" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J46" t="s">
-        <x:v>192</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K46">
         <x:v>37.341022029999998</x:v>
@@ -2776,31 +2777,31 @@
     </x:row>
     <x:row r="47" spans="1:12">
       <x:c r="A47" t="s">
-        <x:v>163</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B47" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C47" t="s">
-        <x:v>171</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D47" t="s">
-        <x:v>180</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E47" t="s">
-        <x:v>43</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F47" t="s">
-        <x:v>199</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="G47" t="s">
-        <x:v>206</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="H47" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I47" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K47">
         <x:v>37.378656040000003</x:v>
@@ -2811,31 +2812,31 @@
     </x:row>
     <x:row r="48" spans="1:12">
       <x:c r="A48" t="s">
-        <x:v>128</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B48" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C48" t="s">
-        <x:v>131</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D48" t="s">
-        <x:v>6</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E48" t="s">
-        <x:v>49</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F48" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G48" t="s">
-        <x:v>222</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="H48" t="s">
-        <x:v>33</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="I48" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K48">
         <x:v>37.38076332</x:v>
@@ -2846,34 +2847,34 @@
     </x:row>
     <x:row r="49" spans="1:12">
       <x:c r="A49" t="s">
-        <x:v>139</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B49" t="s">
-        <x:v>158</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="C49" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D49" t="s">
-        <x:v>105</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E49" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F49" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="G49" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="H49" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I49" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="J49" t="s">
-        <x:v>59</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="K49">
         <x:v>37.436062530000001</x:v>
@@ -2884,31 +2885,31 @@
     </x:row>
     <x:row r="50" spans="1:12">
       <x:c r="A50" t="s">
-        <x:v>144</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B50" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C50" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D50" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="E50" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="D50" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="E50" t="s">
-        <x:v>83</x:v>
-      </x:c>
       <x:c r="F50" t="s">
-        <x:v>210</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G50" t="s">
-        <x:v>217</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="H50" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I50" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K50">
         <x:v>37.405642800000003</x:v>
@@ -2919,31 +2920,31 @@
     </x:row>
     <x:row r="51" spans="1:12">
       <x:c r="A51" t="s">
-        <x:v>120</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B51" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C51" t="s">
-        <x:v>135</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D51" t="s">
-        <x:v>25</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E51" t="s">
-        <x:v>94</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="F51" t="s">
-        <x:v>211</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="G51" t="s">
-        <x:v>221</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H51" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="I51" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="K51">
         <x:v>37.393327390000003</x:v>
@@ -2954,34 +2955,34 @@
     </x:row>
     <x:row r="52" spans="1:12">
       <x:c r="A52" t="s">
-        <x:v>36</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B52" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C52" t="s">
-        <x:v>131</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D52" t="s">
-        <x:v>84</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E52" t="s">
-        <x:v>101</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F52" t="s">
-        <x:v>67</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G52" t="s">
-        <x:v>151</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="H52" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="I52" t="s">
-        <x:v>189</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J52" t="s">
-        <x:v>103</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="K52">
         <x:v>37.36561434</x:v>
@@ -2992,31 +2993,31 @@
     </x:row>
     <x:row r="53" spans="1:12">
       <x:c r="A53" t="s">
-        <x:v>152</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B53" t="s">
-        <x:v>51</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>117</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D53" t="s">
-        <x:v>100</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E53" t="s">
-        <x:v>40</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F53" t="s">
-        <x:v>210</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="G53" t="s">
-        <x:v>215</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="H53" t="s">
-        <x:v>113</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="I53" t="s">
-        <x:v>50</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="K53">
         <x:v>37.365442260000002</x:v>
@@ -3026,7 +3027,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51166665554046630859" footer="0.51166665554046630859"/>
+  <x:pageMargins left="0.74805557727813720703" right="0.74805557727813720703" top="0.98430556058883666992" bottom="0.98430556058883666992" header="0.51152777671813964844" footer="0.51152777671813964844"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="0" fitToHeight="0" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1"/>
 </x:worksheet>

</xml_diff>